<commit_message>
DEV: MPJ_25212 Customer Vendor netting template
git-tfs-id: [https://dev.azure.com/METCASHDevOps]$/Metcash D365 FO Implementation/Trunk/Main;C2664
</commit_message>
<xml_diff>
--- a/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METNettingLineEntryTemplate.xlsx
+++ b/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METNettingLineEntryTemplate.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admind24de965b0\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24300" windowHeight="12495"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24300" windowHeight="12492"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
   <si>
     <t>Journal batch number</t>
   </si>
@@ -116,6 +116,12 @@
   </si>
   <si>
     <t>Netting Line Entry</t>
+  </si>
+  <si>
+    <t>Account dimensions</t>
+  </si>
+  <si>
+    <t>Transaction type</t>
   </si>
 </sst>
 </file>
@@ -305,7 +311,19 @@
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF000000"/>
@@ -490,6 +508,18 @@
       <font>
         <color rgb="FF000000"/>
       </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
       <fill>
         <patternFill patternType="none">
@@ -499,6 +529,54 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -551,54 +629,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -616,49 +646,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A10:S11" insertRow="1" totalsRowShown="0" dataDxfId="26">
-  <autoFilter ref="A10:S11"/>
-  <tableColumns count="19">
-    <tableColumn id="1" name="Date" dataDxfId="15"/>
-    <tableColumn id="4" name="Company" dataDxfId="14"/>
-    <tableColumn id="5" name="Account type" dataDxfId="13"/>
-    <tableColumn id="6" name="Non-ledger account" dataDxfId="12"/>
-    <tableColumn id="7" name="Main account" dataDxfId="11"/>
-    <tableColumn id="8" name="Description" dataDxfId="10"/>
-    <tableColumn id="9" name="Currency" dataDxfId="9"/>
-    <tableColumn id="10" name="Debit" dataDxfId="25"/>
-    <tableColumn id="11" name="Credit" dataDxfId="24"/>
-    <tableColumn id="12" name="Offset company" dataDxfId="8"/>
-    <tableColumn id="17" name="Offset account type" dataDxfId="7"/>
-    <tableColumn id="18" name="Offset Non-ledger account" dataDxfId="6"/>
-    <tableColumn id="2" name="Offset main account" dataDxfId="5"/>
-    <tableColumn id="3" name="Due date" dataDxfId="4"/>
-    <tableColumn id="13" name="Invoice" dataDxfId="3"/>
-    <tableColumn id="14" name="Document date" dataDxfId="2"/>
-    <tableColumn id="15" name="Method of payment" dataDxfId="1"/>
-    <tableColumn id="16" name="Terms of payment" dataDxfId="0"/>
-    <tableColumn id="19" name="Line number" dataDxfId="23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A10:U11" insertRow="1" totalsRowShown="0" dataDxfId="18">
+  <autoFilter ref="A10:U11"/>
+  <tableColumns count="21">
+    <tableColumn id="1" name="Date" dataDxfId="17"/>
+    <tableColumn id="4" name="Company" dataDxfId="16"/>
+    <tableColumn id="5" name="Account type" dataDxfId="15"/>
+    <tableColumn id="6" name="Non-ledger account" dataDxfId="14"/>
+    <tableColumn id="7" name="Account dimensions" dataDxfId="13"/>
+    <tableColumn id="8" name="Main account" dataDxfId="12"/>
+    <tableColumn id="9" name="Description" dataDxfId="11"/>
+    <tableColumn id="10" name="Currency" dataDxfId="10"/>
+    <tableColumn id="11" name="Debit" dataDxfId="21"/>
+    <tableColumn id="12" name="Credit" dataDxfId="20"/>
+    <tableColumn id="17" name="Offset company" dataDxfId="9"/>
+    <tableColumn id="18" name="Offset account type" dataDxfId="8"/>
+    <tableColumn id="2" name="Offset Non-ledger account" dataDxfId="7"/>
+    <tableColumn id="3" name="Offset main account" dataDxfId="6"/>
+    <tableColumn id="13" name="Due date" dataDxfId="5"/>
+    <tableColumn id="14" name="Invoice" dataDxfId="4"/>
+    <tableColumn id="15" name="Document date" dataDxfId="3"/>
+    <tableColumn id="16" name="Method of payment" dataDxfId="2"/>
+    <tableColumn id="19" name="Terms of payment" dataDxfId="1"/>
+    <tableColumn id="20" name="Transaction type" dataDxfId="0"/>
+    <tableColumn id="21" name="Line number" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="A2:B5"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="20"/>
-    <tableColumn id="2" name="Column2" dataDxfId="19"/>
+    <tableColumn id="1" name="Column1" dataDxfId="26"/>
+    <tableColumn id="2" name="Column2" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="D2:D3"/>
   <tableColumns count="1">
-    <tableColumn id="1" name="Column1" dataDxfId="16"/>
+    <tableColumn id="1" name="Column1" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -927,7 +959,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="700" row="1">
+  <wetp:taskpane dockstate="right" visibility="1" width="437" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -938,8 +970,8 @@
   <we:reference id="WA104379629" version="1.3.0.0" store="en-US" storeType="OMEX"/>
   <we:alternateReferences/>
   <we:properties>
+    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev229bdea44aca4237ffdevaos.axcloud.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:false,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1432079768108&quot;,&quot;EntityName&quot;:&quot;LedgerJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;TransDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;Company&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Account dimensions&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityAccountDimension&quot;,&quot;Name&quot;:&quot;DefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Due date&quot;,&quot;LabelId&quot;:&quot;@SYS14588&quot;,&quot;Name&quot;:&quot;DueDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Invoice&quot;,&quot;LabelId&quot;:&quot;@SYS12128&quot;,&quot;Name&quot;:&quot;Invoice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Document date&quot;,&quot;LabelId&quot;:&quot;@SYS2587&quot;,&quot;Name&quot;:&quot;DocumentDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Method of payment&quot;,&quot;LabelId&quot;:&quot;@SYS21698&quot;,&quot;Name&quot;:&quot;PaymentMethod&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Terms of payment&quot;,&quot;LabelId&quot;:&quot;@SYS48&quot;,&quot;Name&quot;:&quot;METPayment&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Transaction type&quot;,&quot;LabelId&quot;:&quot;@SYS21201&quot;,&quot;Name&quot;:&quot;METTransactionType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1432076323970&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076332081&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076337031&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076343437&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1432076322067&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076329093&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076334579&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076341166&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838090160&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalDebit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838095061&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalCredit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1447174003991&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;AccountingCurrency&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;unbound-label-binding-1453226878580&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226925908&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226955011&quot;,&quot;Label&quot;:&quot;Do not change&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:DoNotChange&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311413289&quot;,&quot;Label&quot;:&quot;Journal totals&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalTotals&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311570749&quot;,&quot;Label&quot;:&quot;Netting Line Entry&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalHeader&quot;},{&quot;PublicName&quot;:&quot;LedgerJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;AccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;OffsetAccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;}]}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalLine&quot;,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;Name&quot;:&quot;DimensionCombination&quot;,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{&quot;x-dynint-jobid&quot;:&quot;00000000-0000-0000-0000-000000000000&quot;},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2016-09-19T13:55:41.611Z&quot;,&quot;DocumentId&quot;:&quot;8eceebf9-7bce-4c01-96ff-1b6324908024&quot;,&quot;GenerationActivityId&quot;:&quot;4A056E25-D21E-4624-AD9D-55B4125FBFB8&quot;}"/>
     <we:property name="Features" value="{&quot;LogDomEvents&quot;:false,&quot;LogTelemetry&quot;:true}"/>
-    <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev5336f15c42cfd56dedevaos.cloudax.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:false,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1432079768108&quot;,&quot;EntityName&quot;:&quot;LedgerJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;TransDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;Company&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Due date&quot;,&quot;LabelId&quot;:&quot;@SYS14588&quot;,&quot;Name&quot;:&quot;DueDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Invoice&quot;,&quot;LabelId&quot;:&quot;@SYS12128&quot;,&quot;Name&quot;:&quot;Invoice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Document date&quot;,&quot;LabelId&quot;:&quot;@SYS2587&quot;,&quot;Name&quot;:&quot;DocumentDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Method of payment&quot;,&quot;LabelId&quot;:&quot;@SYS21698&quot;,&quot;Name&quot;:&quot;PaymentMethod&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Terms of payment&quot;,&quot;LabelId&quot;:&quot;@SYS48&quot;,&quot;Name&quot;:&quot;METPayment&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1432076323970&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076332081&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076337031&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076343437&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1432076322067&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076329093&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076334579&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076341166&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838090160&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalDebit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838095061&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalCredit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1447174003991&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;AccountingCurrency&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;unbound-label-binding-1453226878580&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226925908&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226955011&quot;,&quot;Label&quot;:&quot;Do not change&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:DoNotChange&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311413289&quot;,&quot;Label&quot;:&quot;Journal totals&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalTotals&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311570749&quot;,&quot;Label&quot;:&quot;Netting Line Entry&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalHeader&quot;},{&quot;PublicName&quot;:&quot;LedgerJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;AccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;OffsetAccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;}]}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalLine&quot;,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;Name&quot;:&quot;DimensionCombination&quot;,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{&quot;x-dynint-jobid&quot;:&quot;00000000-0000-0000-0000-000000000000&quot;},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2016-09-19T13:55:41.611Z&quot;,&quot;DocumentId&quot;:&quot;8eceebf9-7bce-4c01-96ff-1b6324908024&quot;,&quot;GenerationActivityId&quot;:&quot;4A056E25-D21E-4624-AD9D-55B4125FBFB8&quot;}"/>
   </we:properties>
   <we:bindings>
     <we:binding id="value-binding-1432076322067" type="text" appref="{224939D4-6CDF-464E-819A-7B21F544FA44}"/>
@@ -968,34 +1000,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:U11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.1328125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="11.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.73046875" customWidth="1"/>
-    <col min="4" max="4" width="23.265625" customWidth="1"/>
-    <col min="5" max="5" width="20.73046875" customWidth="1"/>
-    <col min="6" max="7" width="15.73046875" customWidth="1"/>
-    <col min="8" max="8" width="17.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.59765625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.265625" customWidth="1"/>
-    <col min="12" max="12" width="18.3984375" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" style="9" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" customWidth="1"/>
+    <col min="6" max="7" width="15.77734375" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.44140625" customWidth="1"/>
     <col min="13" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="15.1328125" customWidth="1"/>
-    <col min="16" max="16" width="15.9296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.46484375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" customWidth="1"/>
+    <col min="16" max="16" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.9296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.21875" customWidth="1"/>
+    <col min="21" max="21" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:21" ht="21" x14ac:dyDescent="0.4">
       <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:21" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>0</v>
       </c>
@@ -1004,7 +1038,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>1</v>
       </c>
@@ -1013,7 +1047,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>2</v>
       </c>
@@ -1022,7 +1056,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
@@ -1035,7 +1069,7 @@
       </c>
       <c r="G6" s="19"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="E7" s="2"/>
       <c r="F7" s="8" t="s">
         <v>6</v>
@@ -1044,7 +1078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="E8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1056,14 +1090,14 @@
       </c>
       <c r="J8" s="12"/>
     </row>
-    <row r="9" spans="1:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="S9" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>4</v>
       </c>
@@ -1077,52 +1111,58 @@
         <v>23</v>
       </c>
       <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" t="s">
         <v>21</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>5</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>6</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>7</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>9</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>20</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>24</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>22</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>28</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>29</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>26</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>27</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
+        <v>33</v>
+      </c>
+      <c r="U10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="18"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -1130,18 +1170,20 @@
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
-      <c r="H11" s="14"/>
+      <c r="H11" s="13"/>
       <c r="I11" s="14"/>
-      <c r="J11" s="13"/>
+      <c r="J11" s="14"/>
       <c r="K11" s="13"/>
       <c r="L11" s="13"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="18"/>
       <c r="R11" s="13"/>
-      <c r="S11" s="14"/>
+      <c r="S11" s="13"/>
+      <c r="T11" s="13"/>
+      <c r="U11" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1224,20 +1266,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11" style="16" customWidth="1"/>
-    <col min="3" max="3" width="9.1328125" style="16"/>
+    <col min="3" max="3" width="9.109375" style="16"/>
     <col min="4" max="4" width="11" style="16" customWidth="1"/>
-    <col min="5" max="16384" width="9.1328125" style="16"/>
+    <col min="5" max="16384" width="9.109375" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>12</v>
       </c>
@@ -1248,7 +1290,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>15</v>
       </c>
@@ -1256,7 +1298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>25</v>
       </c>
@@ -1264,7 +1306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
DEV:MPJ_25212 Customer Vendor netting template
git-tfs-id: [https://dev.azure.com/METCASHDevOps]$/Metcash D365 FO Implementation/Trunk/Main;C2686
</commit_message>
<xml_diff>
--- a/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METNettingLineEntryTemplate.xlsx
+++ b/Metadata/Metcash/Metcash/AxResource/ResourceContent/Data/METNettingLineEntryTemplate.xlsx
@@ -529,6 +529,62 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF000000"/>
       </font>
@@ -573,62 +629,6 @@
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -646,7 +646,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A10:U11" insertRow="1" totalsRowShown="0" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A10:U11" insertRow="1" totalsRowShown="0" dataDxfId="28">
   <autoFilter ref="A10:U11"/>
   <tableColumns count="21">
     <tableColumn id="1" name="Date" dataDxfId="17"/>
@@ -657,8 +657,8 @@
     <tableColumn id="8" name="Main account" dataDxfId="12"/>
     <tableColumn id="9" name="Description" dataDxfId="11"/>
     <tableColumn id="10" name="Currency" dataDxfId="10"/>
-    <tableColumn id="11" name="Debit" dataDxfId="21"/>
-    <tableColumn id="12" name="Credit" dataDxfId="20"/>
+    <tableColumn id="11" name="Debit" dataDxfId="27"/>
+    <tableColumn id="12" name="Credit" dataDxfId="26"/>
     <tableColumn id="17" name="Offset company" dataDxfId="9"/>
     <tableColumn id="18" name="Offset account type" dataDxfId="8"/>
     <tableColumn id="2" name="Offset Non-ledger account" dataDxfId="7"/>
@@ -669,28 +669,28 @@
     <tableColumn id="16" name="Method of payment" dataDxfId="2"/>
     <tableColumn id="19" name="Terms of payment" dataDxfId="1"/>
     <tableColumn id="20" name="Transaction type" dataDxfId="0"/>
-    <tableColumn id="21" name="Line number" dataDxfId="19"/>
+    <tableColumn id="21" name="Line number" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DataCacheKeyTable" displayName="DataCacheKeyTable" ref="A2:B5" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A2:B5"/>
   <tableColumns count="2">
-    <tableColumn id="1" name="Column1" dataDxfId="26"/>
-    <tableColumn id="2" name="Column2" dataDxfId="25"/>
+    <tableColumn id="1" name="Column1" dataDxfId="22"/>
+    <tableColumn id="2" name="Column2" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataCacheDataTable" displayName="DataCacheDataTable" ref="D2:D3" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="D2:D3"/>
   <tableColumns count="1">
-    <tableColumn id="1" name="Column1" dataDxfId="22"/>
+    <tableColumn id="1" name="Column1" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -959,7 +959,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="437" row="2">
+  <wetp:taskpane dockstate="right" visibility="1" width="437" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -970,8 +970,8 @@
   <we:reference id="WA104379629" version="1.3.0.0" store="en-US" storeType="OMEX"/>
   <we:alternateReferences/>
   <we:properties>
+    <we:property name="Features" value="{&quot;LogDomEvents&quot;:false,&quot;LogTelemetry&quot;:true}"/>
     <we:property name="RuntimeConfig" value="{&quot;Version&quot;:1,&quot;HostName&quot;:&quot;https://metcash-dev229bdea44aca4237ffdevaos.axcloud.dynamics.com&quot;,&quot;DiscoveryServiceLocation&quot;:&quot;&quot;,&quot;NamespaceId&quot;:&quot;&quot;,&quot;Applets&quot;:{&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;:{&quot;DataOptions&quot;:{&quot;AutoSizeColumns&quot;:false,&quot;RefreshOnOpen&quot;:true,&quot;CellRefreshLimit&quot;:1000000,&quot;ConfirmPublishOnCreate&quot;:false,&quot;ConfirmPublishOnUpdate&quot;:false,&quot;ConfirmPublishOnDelete&quot;:true,&quot;PublishSequentially&quot;:true,&quot;EnableDesign&quot;:true,&quot;EnablePublishOrder&quot;:false,&quot;EnvironmentPublishBatchLimit&quot;:100,&quot;WorkbookPublishBatchLimit&quot;:100},&quot;Version&quot;:1,&quot;Bindings&quot;:[{&quot;Id&quot;:&quot;table-binding-1432079768108&quot;,&quot;EntityName&quot;:&quot;LedgerJournalLine&quot;,&quot;Fields&quot;:[{&quot;Label&quot;:&quot;Date&quot;,&quot;LabelId&quot;:&quot;@SYS7402&quot;,&quot;Name&quot;:&quot;TransDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Company&quot;,&quot;LabelId&quot;:&quot;@SYS13342&quot;,&quot;Name&quot;:&quot;Company&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Account type&quot;,&quot;LabelId&quot;:&quot;@SYS27730&quot;,&quot;Name&quot;:&quot;AccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Account dimensions&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalEntityAccountDimension&quot;,&quot;Name&quot;:&quot;DefaultDimensionDisplayValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;AccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Description&quot;,&quot;LabelId&quot;:&quot;@SYS13566&quot;,&quot;Name&quot;:&quot;Text&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Currency&quot;,&quot;LabelId&quot;:&quot;@SYS7572&quot;,&quot;Name&quot;:&quot;CurrencyCode&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS9512&quot;,&quot;Name&quot;:&quot;DebitAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS7084&quot;,&quot;Name&quot;:&quot;CreditAmount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset company&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:OffsetCompany&quot;,&quot;Name&quot;:&quot;OffsetCompany&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset account type&quot;,&quot;LabelId&quot;:&quot;@SYS23950&quot;,&quot;Name&quot;:&quot;OffsetAccountType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Offset Non-ledger account&quot;,&quot;Name&quot;:&quot;AccountValue&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Offset main account&quot;,&quot;Name&quot;:&quot;MainAccount&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false,&quot;EntityName&quot;:&quot;DimensionCombination&quot;,&quot;EntityRelation&quot;:&quot;LedgerJournalLineOffsetLedgerDimensionCombination&quot;,&quot;DisplayValueFieldName&quot;:&quot;OffsetAccountDisplayValue&quot;},{&quot;Label&quot;:&quot;Due date&quot;,&quot;LabelId&quot;:&quot;@SYS14588&quot;,&quot;Name&quot;:&quot;DueDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Invoice&quot;,&quot;LabelId&quot;:&quot;@SYS12128&quot;,&quot;Name&quot;:&quot;Invoice&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Document date&quot;,&quot;LabelId&quot;:&quot;@SYS2587&quot;,&quot;Name&quot;:&quot;DocumentDate&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Method of payment&quot;,&quot;LabelId&quot;:&quot;@SYS21698&quot;,&quot;Name&quot;:&quot;PaymentMethod&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Terms of payment&quot;,&quot;LabelId&quot;:&quot;@SYS48&quot;,&quot;Name&quot;:&quot;METPayment&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Transaction type&quot;,&quot;LabelId&quot;:&quot;@SYS21201&quot;,&quot;Name&quot;:&quot;METTransactionType&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Label&quot;:&quot;Line number&quot;,&quot;LabelId&quot;:&quot;@SYS15682&quot;,&quot;Name&quot;:&quot;LineNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}]}],&quot;LabelBindings&quot;:[{&quot;Id&quot;:&quot;label-binding-1432076323970&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076332081&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076337031&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;label-binding-1432076343437&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;ValueBindings&quot;:[{&quot;Id&quot;:&quot;value-binding-1432076322067&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076329093&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;Description&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076334579&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalName&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1432076341166&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;IsPosted&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838090160&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalDebit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1444838095061&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;JournalTotalCredit&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false},{&quot;Id&quot;:&quot;value-binding-1447174003991&quot;,&quot;EntityName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Field&quot;:&quot;AccountingCurrency&quot;,&quot;ForceReadOnly&quot;:false,&quot;ForceReadOnlyOnCreate&quot;:false}],&quot;UnboundLabelBindings&quot;:[{&quot;Id&quot;:&quot;unbound-label-binding-1453226878580&quot;,&quot;Label&quot;:&quot;Debit&quot;,&quot;LabelId&quot;:&quot;@SYS41268&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226925908&quot;,&quot;Label&quot;:&quot;Credit&quot;,&quot;LabelId&quot;:&quot;@SYS35221&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453226955011&quot;,&quot;Label&quot;:&quot;Do not change&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:DoNotChange&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311413289&quot;,&quot;Label&quot;:&quot;Journal totals&quot;,&quot;LabelId&quot;:&quot;@GeneralLedger:JournalTotals&quot;},{&quot;Id&quot;:&quot;unbound-label-binding-1453311570749&quot;,&quot;Label&quot;:&quot;Netting Line Entry&quot;}],&quot;Entities&quot;:[{&quot;PublicName&quot;:&quot;LedgerJournalHeader&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalHeader&quot;},{&quot;PublicName&quot;:&quot;LedgerJournalLine&quot;,&quot;Filter&quot;:{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;JournalBatchNumber&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;00480&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;dataAreaId&quot;,&quot;Type&quot;:&quot;Edm.String&quot;},&quot;Right&quot;:&quot;usmf&quot;}]},{&quot;Operator&quot;:&quot;and&quot;,&quot;Collection&quot;:[{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;AccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;},{&quot;Operator&quot;:&quot;eq&quot;,&quot;Left&quot;:{&quot;Field&quot;:&quot;OffsetAccountType&quot;,&quot;Type&quot;:&quot;Microsoft.Dynamics.DataEntities.LedgerJournalACType&quot;},&quot;Right&quot;:&quot;Ledger&quot;}]}]},&quot;RefreshAfterPublish&quot;:true,&quot;Name&quot;:&quot;LedgerJournalLine&quot;,&quot;PublishIndex&quot;:0},{&quot;PublicName&quot;:&quot;DimensionCombination&quot;,&quot;RefreshAfterPublish&quot;:false,&quot;Name&quot;:&quot;DimensionCombination&quot;,&quot;PublishIndex&quot;:0}],&quot;SectionBindings&quot;:[]}},&quot;ActiveAppletId&quot;:&quot;Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet&quot;,&quot;Headers&quot;:{&quot;x-dynint-jobid&quot;:&quot;00000000-0000-0000-0000-000000000000&quot;},&quot;Language&quot;:&quot;EN&quot;,&quot;DateCreated&quot;:&quot;2016-09-19T13:55:41.611Z&quot;,&quot;DocumentId&quot;:&quot;8eceebf9-7bce-4c01-96ff-1b6324908024&quot;,&quot;GenerationActivityId&quot;:&quot;4A056E25-D21E-4624-AD9D-55B4125FBFB8&quot;}"/>
-    <we:property name="Features" value="{&quot;LogDomEvents&quot;:false,&quot;LogTelemetry&quot;:true}"/>
   </we:properties>
   <we:bindings>
     <we:binding id="value-binding-1432076322067" type="text" appref="{224939D4-6CDF-464E-819A-7B21F544FA44}"/>
@@ -1093,7 +1093,7 @@
     <row r="9" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="S9" s="17" t="s">
+      <c r="U9" s="17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
     <mergeCell ref="F6:G6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="S9" r:id="rId1" tooltip="Label ID: @GeneralLedger:DoNotChange" display="https://usnconeboxax1aos.cloud.onebox.dynamics.com/OfficeApps/Applets/ExcelDataConnector/Excel.html?AppletID=Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet"/>
+    <hyperlink ref="U9" r:id="rId1" tooltip="Label ID: @GeneralLedger:DoNotChange" display="https://usnconeboxax1aos.cloud.onebox.dynamics.com/OfficeApps/Applets/ExcelDataConnector/Excel.html?AppletID=Microsoft.Dynamics.Platform.Integration.Office.DataConnectorApplet"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>